<commit_message>
Crosswalk rules confirmed: Bilog/Binilog -> Pieces or units everywhere; canonical English wins (Bugkos -> Bundle, Putos -> Pack); Whole (chicken) only for exact translations
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/nsu_rename_crosswalk.xlsx
+++ b/outputs/tables/nsu_rename_crosswalk.xlsx
@@ -535,19 +535,19 @@
         <v>5</v>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -1251,19 +1251,19 @@
         <v>162</v>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -1282,19 +1282,19 @@
         <v>1136</v>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping); 1,136 obs - confirm</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -1464,19 +1464,19 @@
         <v>56</v>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -1495,19 +1495,19 @@
         <v>511</v>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -1532,15 +1532,19 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Bugkos</t>
+          <t>Bundle</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>your entry</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>kept; your earlier Bugkos entry reversed per updated rule (canonical English wins)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1559,15 +1563,19 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Bugkos</t>
+          <t>Bundle</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>kept</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>ref canonical: Bundle (canonical English term wins)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1648,7 +1656,7 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Bugkos</t>
+          <t>Bundle</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1658,7 +1666,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>spelling variant of one bugkos</t>
+          <t>spelling of one bugkos = Bundle (ref canonical)</t>
         </is>
       </c>
     </row>
@@ -2300,19 +2308,19 @@
         <v>88</v>
       </c>
       <c r="D62" s="2" t="inlineStr"/>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>Whole (chicken)</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Pieces or units</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>bilog = whole bird? (ref: 'Bilog nga Manok' = Whole (chicken)); could also be Pieces or units - DECIDE</t>
+          <t>ref sheet: Binilog = Pieces or units; Whole (chicken) reserved for exact translations (Bilog nga Manok etc.)</t>
         </is>
       </c>
     </row>
@@ -2362,19 +2370,19 @@
         <v>234</v>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>Whole (chicken)</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Pieces or units</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>bilog = whole bird? (ref: 'Bilog nga Manok' = Whole (chicken)); could also be Pieces or units - DECIDE</t>
+          <t>ref sheet: Bilog = Pieces or units; Whole (chicken) reserved for exact translations (Bilog nga Manok etc.)</t>
         </is>
       </c>
     </row>
@@ -2393,19 +2401,19 @@
         <v>500</v>
       </c>
       <c r="D65" s="2" t="inlineStr"/>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>translation: putos = pack; NOTE putos dominates here (500 obs vs Packs 55) - keep local term instead?</t>
+          <t>translation: putos = pack (ref canonical, rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -2540,19 +2548,19 @@
         <v>90</v>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -2571,19 +2579,19 @@
         <v>406</v>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -2993,19 +3001,19 @@
         <v>99</v>
       </c>
       <c r="D85" s="2" t="inlineStr"/>
-      <c r="E85" s="3" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -3024,19 +3032,19 @@
         <v>602</v>
       </c>
       <c r="D86" s="2" t="inlineStr"/>
-      <c r="E86" s="3" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -3771,19 +3779,19 @@
         <v>37</v>
       </c>
       <c r="D111" s="2" t="inlineStr"/>
-      <c r="E111" s="3" t="inlineStr">
+      <c r="E111" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -3802,19 +3810,19 @@
         <v>221</v>
       </c>
       <c r="D112" s="2" t="inlineStr"/>
-      <c r="E112" s="3" t="inlineStr">
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -4739,19 +4747,19 @@
         <v>132</v>
       </c>
       <c r="D143" s="2" t="inlineStr"/>
-      <c r="E143" s="3" t="inlineStr">
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F143" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -4770,19 +4778,19 @@
         <v>408</v>
       </c>
       <c r="D144" s="2" t="inlineStr"/>
-      <c r="E144" s="3" t="inlineStr">
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F144" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -5339,19 +5347,19 @@
         <v>491</v>
       </c>
       <c r="D163" s="2" t="inlineStr"/>
-      <c r="E163" s="3" t="inlineStr">
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="F163" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>translation: putos = pack; NOTE putos dominates here (491 obs vs Packs 82) - keep local term instead?</t>
+          <t>translation: putos = pack (ref canonical, rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -5494,19 +5502,19 @@
         <v>42</v>
       </c>
       <c r="D168" s="2" t="inlineStr"/>
-      <c r="E168" s="3" t="inlineStr">
+      <c r="E168" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F168" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Binilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Binilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -5525,19 +5533,19 @@
         <v>232</v>
       </c>
       <c r="D169" s="2" t="inlineStr"/>
-      <c r="E169" s="3" t="inlineStr">
+      <c r="E169" s="2" t="inlineStr">
         <is>
           <t>Pieces or units</t>
         </is>
       </c>
-      <c r="F169" s="3" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>ref sheet: Bilog = Pieces or units (follows your Carrot mapping)</t>
+          <t>ref sheet: Bilog = Pieces or units (rule confirmed)</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5775,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Bugkos kept for Camote tops per your entry (dominant local term).</t>
+          <t>canonical English term wins generally (Bugkos -&gt; Bundle, Putos -&gt; Pack);</t>
         </is>
       </c>
     </row>
@@ -5777,14 +5785,14 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Open per-item decisions flagged in notes: Bilog/Binilog -&gt; Pieces or units (large groups),</t>
+          <t>Confirmed rules: Bilog/Binilog -&gt; Pieces or units within every item; Whole (chicken) only for exact</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Chicken Bilog -&gt; Whole (chicken) vs Pieces or units, Putos-dominant items (Crackers, Processed Meat).</t>
+          <t>whole-chicken translations (Bilog nga Manok); canonical English over dominant local terms.</t>
         </is>
       </c>
     </row>

</xml_diff>